<commit_message>
feat(customer): enhance customer CRUD operations with permissions and audit logging
- Completed customer CRUD functionality with role-based permissions and scope validation.
- Implemented atomic audit logging for customer mutations, ensuring no PII is stored in logs.
- Updated API documentation to reflect changes in customer creation and management processes.
- Added tests to validate new behaviors and constraints in customer service.
- Integrated audit module into customer management for comprehensive tracking of changes.
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -12138,6 +12138,60 @@
         </r>
       </text>
     </comment>
+    <comment ref="A71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
+Hoàn thiện CRUD khách hàng: foundation seed đồng bộ customer.view/customer.manage theo vai trò; tạo hồ sơ độc lập chỉ cho GLOBAL vì phạm vi chi nhánh được suy ra qua đơn hàng; update luôn giữ ít nhất email hoặc SĐT; mutation và audit redacted chạy atomic; Admin đồng bộ cache list/detail và chặn xóa MEMBER.
+Sources: OpenAPI:createAdminCustomer/updateAdminCustomer/deactivateAdminCustomer/activateAdminCustomer/deleteAdminCustomer, source:src/modules/customer/admin-customer.service.ts, source:src/modules/customer/admin-customer.controller.ts, source:src/modules/customer/admin-customer.dto.ts, source:../admin/src/features/customers</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
+Hoàn thiện CRUD khách hàng: foundation seed đồng bộ customer.view/customer.manage theo vai trò; tạo hồ sơ độc lập chỉ cho GLOBAL vì phạm vi chi nhánh được suy ra qua đơn hàng; update luôn giữ ít nhất email hoặc SĐT; mutation và audit redacted chạy atomic; Admin đồng bộ cache list/detail và chặn xóa MEMBER.
+Sources: OpenAPI:createAdminCustomer/updateAdminCustomer/deactivateAdminCustomer/activateAdminCustomer/deleteAdminCustomer, source:src/modules/customer/admin-customer.service.ts, source:src/modules/customer/admin-customer.controller.ts, source:src/modules/customer/admin-customer.dto.ts, source:../admin/src/features/customers</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
+Hoàn thiện CRUD khách hàng: foundation seed đồng bộ customer.view/customer.manage theo vai trò; tạo hồ sơ độc lập chỉ cho GLOBAL vì phạm vi chi nhánh được suy ra qua đơn hàng; update luôn giữ ít nhất email hoặc SĐT; mutation và audit redacted chạy atomic; Admin đồng bộ cache list/detail và chặn xóa MEMBER.
+Sources: OpenAPI:createAdminCustomer/updateAdminCustomer/deactivateAdminCustomer/activateAdminCustomer/deleteAdminCustomer, source:src/modules/customer/admin-customer.service.ts, source:src/modules/customer/admin-customer.controller.ts, source:src/modules/customer/admin-customer.dto.ts, source:../admin/src/features/customers</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
+Hoàn thiện CRUD khách hàng: foundation seed đồng bộ customer.view/customer.manage theo vai trò; tạo hồ sơ độc lập chỉ cho GLOBAL vì phạm vi chi nhánh được suy ra qua đơn hàng; update luôn giữ ít nhất email hoặc SĐT; mutation và audit redacted chạy atomic; Admin đồng bộ cache list/detail và chặn xóa MEMBER.
+Sources: OpenAPI:createAdminCustomer/updateAdminCustomer/deactivateAdminCustomer/activateAdminCustomer/deleteAdminCustomer, source:src/modules/customer/admin-customer.service.ts, source:src/modules/customer/admin-customer.controller.ts, source:src/modules/customer/admin-customer.dto.ts, source:../admin/src/features/customers</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
+Hoàn thiện CRUD khách hàng: foundation seed đồng bộ customer.view/customer.manage theo vai trò; tạo hồ sơ độc lập chỉ cho GLOBAL vì phạm vi chi nhánh được suy ra qua đơn hàng; update luôn giữ ít nhất email hoặc SĐT; mutation và audit redacted chạy atomic; Admin đồng bộ cache list/detail và chặn xóa MEMBER.
+Sources: OpenAPI:createAdminCustomer/updateAdminCustomer/deactivateAdminCustomer/activateAdminCustomer/deleteAdminCustomer, source:src/modules/customer/admin-customer.service.ts, source:src/modules/customer/admin-customer.controller.ts, source:src/modules/customer/admin-customer.dto.ts, source:../admin/src/features/customers</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
+Hoàn thiện CRUD khách hàng: foundation seed đồng bộ customer.view/customer.manage theo vai trò; tạo hồ sơ độc lập chỉ cho GLOBAL vì phạm vi chi nhánh được suy ra qua đơn hàng; update luôn giữ ít nhất email hoặc SĐT; mutation và audit redacted chạy atomic; Admin đồng bộ cache list/detail và chặn xóa MEMBER.
+Sources: OpenAPI:createAdminCustomer/updateAdminCustomer/deactivateAdminCustomer/activateAdminCustomer/deleteAdminCustomer, source:src/modules/customer/admin-customer.service.ts, source:src/modules/customer/admin-customer.controller.ts, source:src/modules/customer/admin-customer.dto.ts, source:../admin/src/features/customers</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -13413,7 +13467,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8180" uniqueCount="1858">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8186" uniqueCount="1863">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -19367,6 +19421,25 @@
 source:src/modules/system/parameters/system-parameter.catalog.ts
 source:src/modules/system/parameters/integration-config.service.ts
 test:src/modules/system/parameters/system-parameter.service.spec.ts</t>
+  </si>
+  <si>
+    <t>API-20260918-CUSTOMER-CRUD-HARDENING</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>CUSTOMER+PERMISSION+AUDIT+ADMIN</t>
+  </si>
+  <si>
+    <t>Hoàn thiện CRUD khách hàng: foundation seed đồng bộ customer.view/customer.manage theo vai trò; tạo hồ sơ độc lập chỉ cho GLOBAL vì phạm vi chi nhánh được suy ra qua đơn hàng; update luôn giữ ít nhất email hoặc SĐT; mutation và audit redacted chạy atomic; Admin đồng bộ cache list/detail và chặn xóa MEMBER.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAPI:createAdminCustomer/updateAdminCustomer/deactivateAdminCustomer/activateAdminCustomer/deleteAdminCustomer
+source:src/modules/customer/admin-customer.service.ts
+source:src/modules/customer/admin-customer.controller.ts
+source:src/modules/customer/admin-customer.dto.ts
+source:../admin/src/features/customers</t>
   </si>
 </sst>
 </file>
@@ -48276,7 +48349,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -49684,6 +49757,26 @@
         <v>1857</v>
       </c>
       <c r="F70" s="6" t="s">
+        <v>1569</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="6" t="s">
+        <v>1858</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>1859</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>1860</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>1861</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>1862</v>
+      </c>
+      <c r="F71" s="6" t="s">
         <v>1569</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update system parameters to allow optional reason for changes while maintaining audit logging
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -12141,13 +12141,121 @@
     <comment ref="A71" authorId="0">
       <text>
         <r>
+          <t xml:space="preserve">API-20260918-CATALOG-READ-PARALLEL · 2026-09-18 · API+PERSISTENCE
+Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
+Sources: OpenAPI:listCatalogProducts/listAdminProducts, source:src/modules/catalog/products/services/products.service.ts, test:src/modules/catalog/products/services/products.service.spec.ts, document:38-api-read-performance-review.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-CATALOG-READ-PARALLEL · 2026-09-18 · API+PERSISTENCE
+Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
+Sources: OpenAPI:listCatalogProducts/listAdminProducts, source:src/modules/catalog/products/services/products.service.ts, test:src/modules/catalog/products/services/products.service.spec.ts, document:38-api-read-performance-review.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-CATALOG-READ-PARALLEL · 2026-09-18 · API+PERSISTENCE
+Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
+Sources: OpenAPI:listCatalogProducts/listAdminProducts, source:src/modules/catalog/products/services/products.service.ts, test:src/modules/catalog/products/services/products.service.spec.ts, document:38-api-read-performance-review.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-CATALOG-READ-PARALLEL · 2026-09-18 · API+PERSISTENCE
+Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
+Sources: OpenAPI:listCatalogProducts/listAdminProducts, source:src/modules/catalog/products/services/products.service.ts, test:src/modules/catalog/products/services/products.service.spec.ts, document:38-api-read-performance-review.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-CATALOG-READ-PARALLEL · 2026-09-18 · API+PERSISTENCE
+Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
+Sources: OpenAPI:listCatalogProducts/listAdminProducts, source:src/modules/catalog/products/services/products.service.ts, test:src/modules/catalog/products/services/products.service.spec.ts, document:38-api-read-performance-review.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-CATALOG-READ-PARALLEL · 2026-09-18 · API+PERSISTENCE
+Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
+Sources: OpenAPI:listCatalogProducts/listAdminProducts, source:src/modules/catalog/products/services/products.service.ts, test:src/modules/catalog/products/services/products.service.spec.ts, document:38-api-read-performance-review.md</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-PARAMETER-OPTIONAL-REASON · 2026-09-18 · API+ADMIN
+Lý do khi sửa/ngừng dùng tham số là tùy chọn; expectedVersion và audit actor/request/thay đổi vẫn bắt buộc. Không thay đổi bảng dữ liệu.
+Sources: OpenAPI:updateAdminSystemParameter/deleteAdminSystemParameter, source:src/modules/system/parameters/system-parameter.service.ts, source:../admin/src/features/system-parameters</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-PARAMETER-OPTIONAL-REASON · 2026-09-18 · API+ADMIN
+Lý do khi sửa/ngừng dùng tham số là tùy chọn; expectedVersion và audit actor/request/thay đổi vẫn bắt buộc. Không thay đổi bảng dữ liệu.
+Sources: OpenAPI:updateAdminSystemParameter/deleteAdminSystemParameter, source:src/modules/system/parameters/system-parameter.service.ts, source:../admin/src/features/system-parameters</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-PARAMETER-OPTIONAL-REASON · 2026-09-18 · API+ADMIN
+Lý do khi sửa/ngừng dùng tham số là tùy chọn; expectedVersion và audit actor/request/thay đổi vẫn bắt buộc. Không thay đổi bảng dữ liệu.
+Sources: OpenAPI:updateAdminSystemParameter/deleteAdminSystemParameter, source:src/modules/system/parameters/system-parameter.service.ts, source:../admin/src/features/system-parameters</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-PARAMETER-OPTIONAL-REASON · 2026-09-18 · API+ADMIN
+Lý do khi sửa/ngừng dùng tham số là tùy chọn; expectedVersion và audit actor/request/thay đổi vẫn bắt buộc. Không thay đổi bảng dữ liệu.
+Sources: OpenAPI:updateAdminSystemParameter/deleteAdminSystemParameter, source:src/modules/system/parameters/system-parameter.service.ts, source:../admin/src/features/system-parameters</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-PARAMETER-OPTIONAL-REASON · 2026-09-18 · API+ADMIN
+Lý do khi sửa/ngừng dùng tham số là tùy chọn; expectedVersion và audit actor/request/thay đổi vẫn bắt buộc. Không thay đổi bảng dữ liệu.
+Sources: OpenAPI:updateAdminSystemParameter/deleteAdminSystemParameter, source:src/modules/system/parameters/system-parameter.service.ts, source:../admin/src/features/system-parameters</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260918-PARAMETER-OPTIONAL-REASON · 2026-09-18 · API+ADMIN
+Lý do khi sửa/ngừng dùng tham số là tùy chọn; expectedVersion và audit actor/request/thay đổi vẫn bắt buộc. Không thay đổi bảng dữ liệu.
+Sources: OpenAPI:updateAdminSystemParameter/deleteAdminSystemParameter, source:src/modules/system/parameters/system-parameter.service.ts, source:../admin/src/features/system-parameters</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A73" authorId="0">
+      <text>
+        <r>
           <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
 Hoàn thiện CRUD khách hàng: foundation seed đồng bộ customer.view/customer.manage theo vai trò; tạo hồ sơ độc lập chỉ cho GLOBAL vì phạm vi chi nhánh được suy ra qua đơn hàng; update luôn giữ ít nhất email hoặc SĐT; mutation và audit redacted chạy atomic; Admin đồng bộ cache list/detail và chặn xóa MEMBER.
 Sources: OpenAPI:createAdminCustomer/updateAdminCustomer/deactivateAdminCustomer/activateAdminCustomer/deleteAdminCustomer, source:src/modules/customer/admin-customer.service.ts, source:src/modules/customer/admin-customer.controller.ts, source:src/modules/customer/admin-customer.dto.ts, source:../admin/src/features/customers</t>
         </r>
       </text>
     </comment>
-    <comment ref="B71" authorId="0">
+    <comment ref="B73" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
@@ -12156,7 +12264,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C71" authorId="0">
+    <comment ref="C73" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
@@ -12165,7 +12273,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D71" authorId="0">
+    <comment ref="D73" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
@@ -12174,7 +12282,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E71" authorId="0">
+    <comment ref="E73" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
@@ -12183,7 +12291,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F71" authorId="0">
+    <comment ref="F73" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
@@ -13467,7 +13575,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8186" uniqueCount="1863">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8198" uniqueCount="1871">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -19423,10 +19531,39 @@
 test:src/modules/system/parameters/system-parameter.service.spec.ts</t>
   </si>
   <si>
+    <t>API-20260918-CATALOG-READ-PARALLEL</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>API+PERSISTENCE</t>
+  </si>
+  <si>
+    <t>Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAPI:listCatalogProducts/listAdminProducts
+source:src/modules/catalog/products/services/products.service.ts
+test:src/modules/catalog/products/services/products.service.spec.ts
+document:38-api-read-performance-review.md</t>
+  </si>
+  <si>
+    <t>API-20260918-PARAMETER-OPTIONAL-REASON</t>
+  </si>
+  <si>
+    <t>API+ADMIN</t>
+  </si>
+  <si>
+    <t>Lý do khi sửa/ngừng dùng tham số là tùy chọn; expectedVersion và audit actor/request/thay đổi vẫn bắt buộc. Không thay đổi bảng dữ liệu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAPI:updateAdminSystemParameter/deleteAdminSystemParameter
+source:src/modules/system/parameters/system-parameter.service.ts
+source:../admin/src/features/system-parameters</t>
+  </si>
+  <si>
     <t>API-20260918-CUSTOMER-CRUD-HARDENING</t>
-  </si>
-  <si>
-    <t>2026-09-18</t>
   </si>
   <si>
     <t>CUSTOMER+PERMISSION+AUDIT+ADMIN</t>
@@ -48349,7 +48486,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F73"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -49777,6 +49914,46 @@
         <v>1862</v>
       </c>
       <c r="F71" s="6" t="s">
+        <v>1569</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="6" t="s">
+        <v>1863</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>1859</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>1864</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>1865</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>1866</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>1569</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="6" t="s">
+        <v>1867</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>1859</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>1868</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>1869</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>1870</v>
+      </c>
+      <c r="F73" s="6" t="s">
         <v>1569</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: enhance role lifecycle management and update related documentation
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -12141,58 +12141,166 @@
     <comment ref="A71" authorId="0">
       <text>
         <r>
+          <t xml:space="preserve">API-20260919-ADMIN-REFRESH-RECOVERY · 2026-09-19 · AUTH+API+ADMIN
+Production refresh cookie hỗ trợ request cross-site bằng SameSite=None/Secure; Admin giữ access token trong memory, tự dọn phiên/cache, redirect login và toast một lần khi refresh thất bại. Không thay đổi database.
+Sources: OpenAPI:refreshAdminToken/getAdminCurrentUser, source:src/modules/auth/auth-token-transport.service.ts, source:../admin/src/core/auth, test:src/modules/auth/auth-token-transport.service.spec.ts, test:../admin/src/lib/api/fetcher.test.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260919-ADMIN-REFRESH-RECOVERY · 2026-09-19 · AUTH+API+ADMIN
+Production refresh cookie hỗ trợ request cross-site bằng SameSite=None/Secure; Admin giữ access token trong memory, tự dọn phiên/cache, redirect login và toast một lần khi refresh thất bại. Không thay đổi database.
+Sources: OpenAPI:refreshAdminToken/getAdminCurrentUser, source:src/modules/auth/auth-token-transport.service.ts, source:../admin/src/core/auth, test:src/modules/auth/auth-token-transport.service.spec.ts, test:../admin/src/lib/api/fetcher.test.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260919-ADMIN-REFRESH-RECOVERY · 2026-09-19 · AUTH+API+ADMIN
+Production refresh cookie hỗ trợ request cross-site bằng SameSite=None/Secure; Admin giữ access token trong memory, tự dọn phiên/cache, redirect login và toast một lần khi refresh thất bại. Không thay đổi database.
+Sources: OpenAPI:refreshAdminToken/getAdminCurrentUser, source:src/modules/auth/auth-token-transport.service.ts, source:../admin/src/core/auth, test:src/modules/auth/auth-token-transport.service.spec.ts, test:../admin/src/lib/api/fetcher.test.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260919-ADMIN-REFRESH-RECOVERY · 2026-09-19 · AUTH+API+ADMIN
+Production refresh cookie hỗ trợ request cross-site bằng SameSite=None/Secure; Admin giữ access token trong memory, tự dọn phiên/cache, redirect login và toast một lần khi refresh thất bại. Không thay đổi database.
+Sources: OpenAPI:refreshAdminToken/getAdminCurrentUser, source:src/modules/auth/auth-token-transport.service.ts, source:../admin/src/core/auth, test:src/modules/auth/auth-token-transport.service.spec.ts, test:../admin/src/lib/api/fetcher.test.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260919-ADMIN-REFRESH-RECOVERY · 2026-09-19 · AUTH+API+ADMIN
+Production refresh cookie hỗ trợ request cross-site bằng SameSite=None/Secure; Admin giữ access token trong memory, tự dọn phiên/cache, redirect login và toast một lần khi refresh thất bại. Không thay đổi database.
+Sources: OpenAPI:refreshAdminToken/getAdminCurrentUser, source:src/modules/auth/auth-token-transport.service.ts, source:../admin/src/core/auth, test:src/modules/auth/auth-token-transport.service.spec.ts, test:../admin/src/lib/api/fetcher.test.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F71" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260919-ADMIN-REFRESH-RECOVERY · 2026-09-19 · AUTH+API+ADMIN
+Production refresh cookie hỗ trợ request cross-site bằng SameSite=None/Secure; Admin giữ access token trong memory, tự dọn phiên/cache, redirect login và toast một lần khi refresh thất bại. Không thay đổi database.
+Sources: OpenAPI:refreshAdminToken/getAdminCurrentUser, source:src/modules/auth/auth-token-transport.service.ts, source:../admin/src/core/auth, test:src/modules/auth/auth-token-transport.service.spec.ts, test:../admin/src/lib/api/fetcher.test.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260919-SYSTEM-ROLE-LIFECYCLE · 2026-09-19 · IAM+API+ADMIN
+OWNER tiếp tục bất biến. DELETE BRANCH_MANAGER/STAFF chuyển vai trò sang INACTIVE, tăng permission_version của người đang được gán và giữ lịch sử; custom role chưa gán mới xóa vật lý. Foundation seed chỉ bootstrap role còn thiếu và không ghi đè tên, trạng thái hoặc tập quyền do Admin đã chỉnh. Không thay đổi schema database.
+Sources: OpenAPI:updateAdminRole/deleteAdminRole, source:src/modules/iam/iam.service.ts, source:src/modules/iam/prisma-iam.repository.ts, source:prisma/seed.ts, source:../admin/src/features/roles, test:src/modules/iam/iam.role-administration.spec.ts, test:src/modules/iam/prisma-iam.role-status.spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260919-SYSTEM-ROLE-LIFECYCLE · 2026-09-19 · IAM+API+ADMIN
+OWNER tiếp tục bất biến. DELETE BRANCH_MANAGER/STAFF chuyển vai trò sang INACTIVE, tăng permission_version của người đang được gán và giữ lịch sử; custom role chưa gán mới xóa vật lý. Foundation seed chỉ bootstrap role còn thiếu và không ghi đè tên, trạng thái hoặc tập quyền do Admin đã chỉnh. Không thay đổi schema database.
+Sources: OpenAPI:updateAdminRole/deleteAdminRole, source:src/modules/iam/iam.service.ts, source:src/modules/iam/prisma-iam.repository.ts, source:prisma/seed.ts, source:../admin/src/features/roles, test:src/modules/iam/iam.role-administration.spec.ts, test:src/modules/iam/prisma-iam.role-status.spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260919-SYSTEM-ROLE-LIFECYCLE · 2026-09-19 · IAM+API+ADMIN
+OWNER tiếp tục bất biến. DELETE BRANCH_MANAGER/STAFF chuyển vai trò sang INACTIVE, tăng permission_version của người đang được gán và giữ lịch sử; custom role chưa gán mới xóa vật lý. Foundation seed chỉ bootstrap role còn thiếu và không ghi đè tên, trạng thái hoặc tập quyền do Admin đã chỉnh. Không thay đổi schema database.
+Sources: OpenAPI:updateAdminRole/deleteAdminRole, source:src/modules/iam/iam.service.ts, source:src/modules/iam/prisma-iam.repository.ts, source:prisma/seed.ts, source:../admin/src/features/roles, test:src/modules/iam/iam.role-administration.spec.ts, test:src/modules/iam/prisma-iam.role-status.spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260919-SYSTEM-ROLE-LIFECYCLE · 2026-09-19 · IAM+API+ADMIN
+OWNER tiếp tục bất biến. DELETE BRANCH_MANAGER/STAFF chuyển vai trò sang INACTIVE, tăng permission_version của người đang được gán và giữ lịch sử; custom role chưa gán mới xóa vật lý. Foundation seed chỉ bootstrap role còn thiếu và không ghi đè tên, trạng thái hoặc tập quyền do Admin đã chỉnh. Không thay đổi schema database.
+Sources: OpenAPI:updateAdminRole/deleteAdminRole, source:src/modules/iam/iam.service.ts, source:src/modules/iam/prisma-iam.repository.ts, source:prisma/seed.ts, source:../admin/src/features/roles, test:src/modules/iam/iam.role-administration.spec.ts, test:src/modules/iam/prisma-iam.role-status.spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260919-SYSTEM-ROLE-LIFECYCLE · 2026-09-19 · IAM+API+ADMIN
+OWNER tiếp tục bất biến. DELETE BRANCH_MANAGER/STAFF chuyển vai trò sang INACTIVE, tăng permission_version của người đang được gán và giữ lịch sử; custom role chưa gán mới xóa vật lý. Foundation seed chỉ bootstrap role còn thiếu và không ghi đè tên, trạng thái hoặc tập quyền do Admin đã chỉnh. Không thay đổi schema database.
+Sources: OpenAPI:updateAdminRole/deleteAdminRole, source:src/modules/iam/iam.service.ts, source:src/modules/iam/prisma-iam.repository.ts, source:prisma/seed.ts, source:../admin/src/features/roles, test:src/modules/iam/iam.role-administration.spec.ts, test:src/modules/iam/prisma-iam.role-status.spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F72" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260919-SYSTEM-ROLE-LIFECYCLE · 2026-09-19 · IAM+API+ADMIN
+OWNER tiếp tục bất biến. DELETE BRANCH_MANAGER/STAFF chuyển vai trò sang INACTIVE, tăng permission_version của người đang được gán và giữ lịch sử; custom role chưa gán mới xóa vật lý. Foundation seed chỉ bootstrap role còn thiếu và không ghi đè tên, trạng thái hoặc tập quyền do Admin đã chỉnh. Không thay đổi schema database.
+Sources: OpenAPI:updateAdminRole/deleteAdminRole, source:src/modules/iam/iam.service.ts, source:src/modules/iam/prisma-iam.repository.ts, source:prisma/seed.ts, source:../admin/src/features/roles, test:src/modules/iam/iam.role-administration.spec.ts, test:src/modules/iam/prisma-iam.role-status.spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A73" authorId="0">
+      <text>
+        <r>
           <t xml:space="preserve">API-20260918-CATALOG-READ-PARALLEL · 2026-09-18 · API+PERSISTENCE
-Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
+Hai phép đọc danh sách sản phẩm và SKU (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
 Sources: OpenAPI:listCatalogProducts/listAdminProducts, source:src/modules/catalog/products/services/products.service.ts, test:src/modules/catalog/products/services/products.service.spec.ts, document:38-api-read-performance-review.md</t>
         </r>
       </text>
     </comment>
-    <comment ref="B71" authorId="0">
+    <comment ref="B73" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CATALOG-READ-PARALLEL · 2026-09-18 · API+PERSISTENCE
-Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
+Hai phép đọc danh sách sản phẩm và SKU (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
 Sources: OpenAPI:listCatalogProducts/listAdminProducts, source:src/modules/catalog/products/services/products.service.ts, test:src/modules/catalog/products/services/products.service.spec.ts, document:38-api-read-performance-review.md</t>
         </r>
       </text>
     </comment>
-    <comment ref="C71" authorId="0">
+    <comment ref="C73" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CATALOG-READ-PARALLEL · 2026-09-18 · API+PERSISTENCE
-Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
+Hai phép đọc danh sách sản phẩm và SKU (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
 Sources: OpenAPI:listCatalogProducts/listAdminProducts, source:src/modules/catalog/products/services/products.service.ts, test:src/modules/catalog/products/services/products.service.spec.ts, document:38-api-read-performance-review.md</t>
         </r>
       </text>
     </comment>
-    <comment ref="D71" authorId="0">
+    <comment ref="D73" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CATALOG-READ-PARALLEL · 2026-09-18 · API+PERSISTENCE
-Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
+Hai phép đọc danh sách sản phẩm và SKU (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
 Sources: OpenAPI:listCatalogProducts/listAdminProducts, source:src/modules/catalog/products/services/products.service.ts, test:src/modules/catalog/products/services/products.service.spec.ts, document:38-api-read-performance-review.md</t>
         </r>
       </text>
     </comment>
-    <comment ref="E71" authorId="0">
+    <comment ref="E73" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CATALOG-READ-PARALLEL · 2026-09-18 · API+PERSISTENCE
-Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
+Hai phép đọc danh sách sản phẩm và SKU (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
 Sources: OpenAPI:listCatalogProducts/listAdminProducts, source:src/modules/catalog/products/services/products.service.ts, test:src/modules/catalog/products/services/products.service.spec.ts, document:38-api-read-performance-review.md</t>
         </r>
       </text>
     </comment>
-    <comment ref="F71" authorId="0">
+    <comment ref="F73" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CATALOG-READ-PARALLEL · 2026-09-18 · API+PERSISTENCE
-Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
+Hai phép đọc danh sách sản phẩm và SKU (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.
 Sources: OpenAPI:listCatalogProducts/listAdminProducts, source:src/modules/catalog/products/services/products.service.ts, test:src/modules/catalog/products/services/products.service.spec.ts, document:38-api-read-performance-review.md</t>
         </r>
       </text>
     </comment>
-    <comment ref="A72" authorId="0">
+    <comment ref="A74" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-PARAMETER-OPTIONAL-REASON · 2026-09-18 · API+ADMIN
@@ -12201,7 +12309,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B72" authorId="0">
+    <comment ref="B74" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-PARAMETER-OPTIONAL-REASON · 2026-09-18 · API+ADMIN
@@ -12210,7 +12318,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C72" authorId="0">
+    <comment ref="C74" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-PARAMETER-OPTIONAL-REASON · 2026-09-18 · API+ADMIN
@@ -12219,7 +12327,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D72" authorId="0">
+    <comment ref="D74" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-PARAMETER-OPTIONAL-REASON · 2026-09-18 · API+ADMIN
@@ -12228,7 +12336,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E72" authorId="0">
+    <comment ref="E74" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-PARAMETER-OPTIONAL-REASON · 2026-09-18 · API+ADMIN
@@ -12237,7 +12345,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F72" authorId="0">
+    <comment ref="F74" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-PARAMETER-OPTIONAL-REASON · 2026-09-18 · API+ADMIN
@@ -12246,7 +12354,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A73" authorId="0">
+    <comment ref="A75" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
@@ -12255,7 +12363,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B73" authorId="0">
+    <comment ref="B75" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
@@ -12264,7 +12372,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C73" authorId="0">
+    <comment ref="C75" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
@@ -12273,7 +12381,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D73" authorId="0">
+    <comment ref="D75" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
@@ -12282,7 +12390,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E73" authorId="0">
+    <comment ref="E75" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
@@ -12291,7 +12399,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F73" authorId="0">
+    <comment ref="F75" authorId="0">
       <text>
         <r>
           <t xml:space="preserve">API-20260918-CUSTOMER-CRUD-HARDENING · 2026-09-18 · CUSTOMER+PERMISSION+AUDIT+ADMIN
@@ -13575,7 +13683,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8198" uniqueCount="1871">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8210" uniqueCount="1880">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -19531,6 +19639,43 @@
 test:src/modules/system/parameters/system-parameter.service.spec.ts</t>
   </si>
   <si>
+    <t>API-20260919-ADMIN-REFRESH-RECOVERY</t>
+  </si>
+  <si>
+    <t>2026-09-19</t>
+  </si>
+  <si>
+    <t>AUTH+API+ADMIN</t>
+  </si>
+  <si>
+    <t>Production refresh cookie hỗ trợ request cross-site bằng SameSite=None/Secure; Admin giữ access token trong memory, tự dọn phiên/cache, redirect login và toast một lần khi refresh thất bại. Không thay đổi database.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAPI:refreshAdminToken/getAdminCurrentUser
+source:src/modules/auth/auth-token-transport.service.ts
+source:../admin/src/core/auth
+test:src/modules/auth/auth-token-transport.service.spec.ts
+test:../admin/src/lib/api/fetcher.test.ts</t>
+  </si>
+  <si>
+    <t>API-20260919-SYSTEM-ROLE-LIFECYCLE</t>
+  </si>
+  <si>
+    <t>IAM+API+ADMIN</t>
+  </si>
+  <si>
+    <t>OWNER tiếp tục bất biến. DELETE BRANCH_MANAGER/STAFF chuyển vai trò sang INACTIVE, tăng permission_version của người đang được gán và giữ lịch sử; custom role chưa gán mới xóa vật lý. Foundation seed chỉ bootstrap role còn thiếu và không ghi đè tên, trạng thái hoặc tập quyền do Admin đã chỉnh. Không thay đổi schema database.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAPI:updateAdminRole/deleteAdminRole
+source:src/modules/iam/iam.service.ts
+source:src/modules/iam/prisma-iam.repository.ts
+source:prisma/seed.ts
+source:../admin/src/features/roles
+test:src/modules/iam/iam.role-administration.spec.ts
+test:src/modules/iam/prisma-iam.role-status.spec.ts</t>
+  </si>
+  <si>
     <t>API-20260918-CATALOG-READ-PARALLEL</t>
   </si>
   <si>
@@ -19540,7 +19685,7 @@
     <t>API+PERSISTENCE</t>
   </si>
   <si>
-    <t>Hai phép đọc danh sách sản phẩm (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.</t>
+    <t>Hai phép đọc danh sách sản phẩm và SKU (findMany/count) chạy song song thay vì mở transaction đọc; response contract và schema không đổi. Theo dõi TTFB và slow query sau deploy.</t>
   </si>
   <si>
     <t xml:space="preserve">OpenAPI:listCatalogProducts/listAdminProducts
@@ -48486,7 +48631,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -49942,18 +50087,58 @@
         <v>1867</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>1859</v>
+        <v>1868</v>
       </c>
       <c r="C73" s="6" t="s">
+        <v>1869</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>1870</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>1871</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>1569</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="6" t="s">
+        <v>1872</v>
+      </c>
+      <c r="B74" s="6" t="s">
         <v>1868</v>
       </c>
-      <c r="D73" s="6" t="s">
-        <v>1869</v>
-      </c>
-      <c r="E73" s="6" t="s">
-        <v>1870</v>
-      </c>
-      <c r="F73" s="6" t="s">
+      <c r="C74" s="6" t="s">
+        <v>1873</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>1874</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>1875</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>1569</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="6" t="s">
+        <v>1876</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>1868</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>1877</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>1878</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>1879</v>
+      </c>
+      <c r="F75" s="6" t="s">
         <v>1569</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement atomic product creation with initial SKU variants
- Added support for creating a product along with its initial SKU variants in a single transaction.
- Updated CreateProductDto to include a variants array with validation for a minimum of 1 and a maximum of 50 variants.
- Enhanced API documentation to reflect new error responses (400, 409, 422) and updated operation summaries.
- Created a new CreateVariantDto for SKU variant details.
- Implemented unit tests for CreateProductDto to validate variant requirements.
- Updated ProductsService to handle the creation of products and variants atomically, ensuring rollback on errors.
- Added README documentation for the Catalog Products module detailing the new functionality and workflow.
- Updated IAM module to enforce security invariants for the OWNER role.
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -12408,6 +12408,60 @@
         </r>
       </text>
     </comment>
+    <comment ref="A76" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260920-PRODUCT-AGGREGATE-CREATE · 2026-09-20 · CATALOG+API+ADMIN
+createAdminProduct bắt buộc nhận 1-50 initial variants và tạo Product, category links, SKU cùng audit trong một Prisma transaction. Admin dùng một form Product + biến thể; endpoint thêm SKU riêng vẫn giữ cho chỉnh sửa sau create. Không thay đổi schema database.
+Sources: OpenAPI:createAdminProduct, source:src/modules/catalog/products/dto/product.dto.ts, source:src/modules/catalog/products/services/products.service.ts, source:../admin/src/features/products</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B76" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260920-PRODUCT-AGGREGATE-CREATE · 2026-09-20 · CATALOG+API+ADMIN
+createAdminProduct bắt buộc nhận 1-50 initial variants và tạo Product, category links, SKU cùng audit trong một Prisma transaction. Admin dùng một form Product + biến thể; endpoint thêm SKU riêng vẫn giữ cho chỉnh sửa sau create. Không thay đổi schema database.
+Sources: OpenAPI:createAdminProduct, source:src/modules/catalog/products/dto/product.dto.ts, source:src/modules/catalog/products/services/products.service.ts, source:../admin/src/features/products</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C76" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260920-PRODUCT-AGGREGATE-CREATE · 2026-09-20 · CATALOG+API+ADMIN
+createAdminProduct bắt buộc nhận 1-50 initial variants và tạo Product, category links, SKU cùng audit trong một Prisma transaction. Admin dùng một form Product + biến thể; endpoint thêm SKU riêng vẫn giữ cho chỉnh sửa sau create. Không thay đổi schema database.
+Sources: OpenAPI:createAdminProduct, source:src/modules/catalog/products/dto/product.dto.ts, source:src/modules/catalog/products/services/products.service.ts, source:../admin/src/features/products</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D76" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260920-PRODUCT-AGGREGATE-CREATE · 2026-09-20 · CATALOG+API+ADMIN
+createAdminProduct bắt buộc nhận 1-50 initial variants và tạo Product, category links, SKU cùng audit trong một Prisma transaction. Admin dùng một form Product + biến thể; endpoint thêm SKU riêng vẫn giữ cho chỉnh sửa sau create. Không thay đổi schema database.
+Sources: OpenAPI:createAdminProduct, source:src/modules/catalog/products/dto/product.dto.ts, source:src/modules/catalog/products/services/products.service.ts, source:../admin/src/features/products</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E76" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260920-PRODUCT-AGGREGATE-CREATE · 2026-09-20 · CATALOG+API+ADMIN
+createAdminProduct bắt buộc nhận 1-50 initial variants và tạo Product, category links, SKU cùng audit trong một Prisma transaction. Admin dùng một form Product + biến thể; endpoint thêm SKU riêng vẫn giữ cho chỉnh sửa sau create. Không thay đổi schema database.
+Sources: OpenAPI:createAdminProduct, source:src/modules/catalog/products/dto/product.dto.ts, source:src/modules/catalog/products/services/products.service.ts, source:../admin/src/features/products</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F76" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260920-PRODUCT-AGGREGATE-CREATE · 2026-09-20 · CATALOG+API+ADMIN
+createAdminProduct bắt buộc nhận 1-50 initial variants và tạo Product, category links, SKU cùng audit trong một Prisma transaction. Admin dùng một form Product + biến thể; endpoint thêm SKU riêng vẫn giữ cho chỉnh sửa sau create. Không thay đổi schema database.
+Sources: OpenAPI:createAdminProduct, source:src/modules/catalog/products/dto/product.dto.ts, source:src/modules/catalog/products/services/products.service.ts, source:../admin/src/features/products</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -13683,7 +13737,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8210" uniqueCount="1880">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8216" uniqueCount="1885">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -19722,6 +19776,24 @@
 source:src/modules/customer/admin-customer.controller.ts
 source:src/modules/customer/admin-customer.dto.ts
 source:../admin/src/features/customers</t>
+  </si>
+  <si>
+    <t>API-20260920-PRODUCT-AGGREGATE-CREATE</t>
+  </si>
+  <si>
+    <t>2026-09-20</t>
+  </si>
+  <si>
+    <t>CATALOG+API+ADMIN</t>
+  </si>
+  <si>
+    <t>createAdminProduct bắt buộc nhận 1-50 initial variants và tạo Product, category links, SKU cùng audit trong một Prisma transaction. Admin dùng một form Product + biến thể; endpoint thêm SKU riêng vẫn giữ cho chỉnh sửa sau create. Không thay đổi schema database.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAPI:createAdminProduct
+source:src/modules/catalog/products/dto/product.dto.ts
+source:src/modules/catalog/products/services/products.service.ts
+source:../admin/src/features/products</t>
   </si>
 </sst>
 </file>
@@ -48631,7 +48703,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -50139,6 +50211,26 @@
         <v>1879</v>
       </c>
       <c r="F75" s="6" t="s">
+        <v>1569</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="6" t="s">
+        <v>1880</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>1881</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>1882</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>1883</v>
+      </c>
+      <c r="E76" s="6" t="s">
+        <v>1884</v>
+      </c>
+      <c r="F76" s="6" t="s">
         <v>1569</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(auth): implement remember-me functionality for refresh tokens
</commit_message>
<xml_diff>
--- a/document/DCTD-UTC-V1-database-model-review.xlsx
+++ b/document/DCTD-UTC-V1-database-model-review.xlsx
@@ -12579,6 +12579,60 @@
         </r>
       </text>
     </comment>
+    <comment ref="A79" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260921-AUTH-REMEMBER-ME · 2026-09-21 · AUTH+API+ADMIN+STOREFRONT
+Login contract nhận rememberMe. COOKIE transport tạo session refresh cookie khi false và persistent refresh cookie theo JWT_REFRESH_TTL_SECONDS khi true; preference HttpOnly theo audience giữ semantics qua refresh rotation và được xóa khi logout. Không thay đổi schema database hoặc thời hạn auth_sessions.
+Sources: OpenAPI:loginAdmin, OpenAPI:loginCustomer, source:src/modules/auth/auth-token-transport.service.ts, test:src/modules/auth/auth-token-transport.service.spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B79" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260921-AUTH-REMEMBER-ME · 2026-09-21 · AUTH+API+ADMIN+STOREFRONT
+Login contract nhận rememberMe. COOKIE transport tạo session refresh cookie khi false và persistent refresh cookie theo JWT_REFRESH_TTL_SECONDS khi true; preference HttpOnly theo audience giữ semantics qua refresh rotation và được xóa khi logout. Không thay đổi schema database hoặc thời hạn auth_sessions.
+Sources: OpenAPI:loginAdmin, OpenAPI:loginCustomer, source:src/modules/auth/auth-token-transport.service.ts, test:src/modules/auth/auth-token-transport.service.spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C79" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260921-AUTH-REMEMBER-ME · 2026-09-21 · AUTH+API+ADMIN+STOREFRONT
+Login contract nhận rememberMe. COOKIE transport tạo session refresh cookie khi false và persistent refresh cookie theo JWT_REFRESH_TTL_SECONDS khi true; preference HttpOnly theo audience giữ semantics qua refresh rotation và được xóa khi logout. Không thay đổi schema database hoặc thời hạn auth_sessions.
+Sources: OpenAPI:loginAdmin, OpenAPI:loginCustomer, source:src/modules/auth/auth-token-transport.service.ts, test:src/modules/auth/auth-token-transport.service.spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D79" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260921-AUTH-REMEMBER-ME · 2026-09-21 · AUTH+API+ADMIN+STOREFRONT
+Login contract nhận rememberMe. COOKIE transport tạo session refresh cookie khi false và persistent refresh cookie theo JWT_REFRESH_TTL_SECONDS khi true; preference HttpOnly theo audience giữ semantics qua refresh rotation và được xóa khi logout. Không thay đổi schema database hoặc thời hạn auth_sessions.
+Sources: OpenAPI:loginAdmin, OpenAPI:loginCustomer, source:src/modules/auth/auth-token-transport.service.ts, test:src/modules/auth/auth-token-transport.service.spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E79" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260921-AUTH-REMEMBER-ME · 2026-09-21 · AUTH+API+ADMIN+STOREFRONT
+Login contract nhận rememberMe. COOKIE transport tạo session refresh cookie khi false và persistent refresh cookie theo JWT_REFRESH_TTL_SECONDS khi true; preference HttpOnly theo audience giữ semantics qua refresh rotation và được xóa khi logout. Không thay đổi schema database hoặc thời hạn auth_sessions.
+Sources: OpenAPI:loginAdmin, OpenAPI:loginCustomer, source:src/modules/auth/auth-token-transport.service.ts, test:src/modules/auth/auth-token-transport.service.spec.ts</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F79" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">API-20260921-AUTH-REMEMBER-ME · 2026-09-21 · AUTH+API+ADMIN+STOREFRONT
+Login contract nhận rememberMe. COOKIE transport tạo session refresh cookie khi false và persistent refresh cookie theo JWT_REFRESH_TTL_SECONDS khi true; preference HttpOnly theo audience giữ semantics qua refresh rotation và được xóa khi logout. Không thay đổi schema database hoặc thời hạn auth_sessions.
+Sources: OpenAPI:loginAdmin, OpenAPI:loginCustomer, source:src/modules/auth/auth-token-transport.service.ts, test:src/modules/auth/auth-token-transport.service.spec.ts</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -13854,7 +13908,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8229" uniqueCount="1896">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8235" uniqueCount="1900">
   <si>
     <t>Hạng mục</t>
   </si>
@@ -19953,6 +20007,21 @@
 source:src/modules/inventory/inventory.constants.ts
 test:src/modules/inventory/inventory.service.spec.ts
 document:src/modules/inventory/README.md</t>
+  </si>
+  <si>
+    <t>API-20260921-AUTH-REMEMBER-ME</t>
+  </si>
+  <si>
+    <t>AUTH+API+ADMIN+STOREFRONT</t>
+  </si>
+  <si>
+    <t>Login contract nhận rememberMe. COOKIE transport tạo session refresh cookie khi false và persistent refresh cookie theo JWT_REFRESH_TTL_SECONDS khi true; preference HttpOnly theo audience giữ semantics qua refresh rotation và được xóa khi logout. Không thay đổi schema database hoặc thời hạn auth_sessions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAPI:loginAdmin
+OpenAPI:loginCustomer
+source:src/modules/auth/auth-token-transport.service.ts
+test:src/modules/auth/auth-token-transport.service.spec.ts</t>
   </si>
 </sst>
 </file>
@@ -48864,7 +48933,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -50432,6 +50501,26 @@
         <v>1895</v>
       </c>
       <c r="F78" s="6" t="s">
+        <v>1570</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="6" t="s">
+        <v>1896</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>1887</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>1897</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>1898</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>1899</v>
+      </c>
+      <c r="F79" s="6" t="s">
         <v>1570</v>
       </c>
     </row>

</xml_diff>